<commit_message>
Update Meta ad data and normalize numeric columns
</commit_message>
<xml_diff>
--- a/data/monthly/【2025年10月】月次数値.xlsx
+++ b/data/monthly/【2025年10月】月次数値.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <fileVersion appName="xl" lastEdited="4" lowestEdited="4" rupBuild="4505"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9302"/>
   <workbookPr codeName="ThisWorkbook"/>
   <bookViews>
-    <workbookView activeTab="0" autoFilterDateGrouping="1" firstSheet="0" minimized="0" showHorizontalScroll="1" showSheetTabs="1" showVerticalScroll="1" tabRatio="600" visibility="visible"/>
+    <workbookView xWindow="420" yWindow="540" windowWidth="11232" windowHeight="3468"/>
   </bookViews>
   <sheets>
-    <sheet name="Worksheet" sheetId="1" r:id="rId4"/>
+    <sheet name="Worksheet" sheetId="1" r:id="rId1"/>
   </sheets>
-  <definedNames/>
-  <calcPr calcId="999999" calcMode="auto" calcCompleted="0" fullCalcOnLoad="1"/>
+  <calcPr calcId="144525"/>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" uniqueCount="54">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="269" uniqueCount="85">
   <si>
     <t>レポート開始日</t>
   </si>
@@ -183,31 +182,122 @@
   </si>
   <si>
     <t>2026-10-30</t>
+  </si>
+  <si>
+    <t>2026-10-01</t>
+  </si>
+  <si>
+    <t>すがや歯科クリニック</t>
+  </si>
+  <si>
+    <t>2026-09-28</t>
+  </si>
+  <si>
+    <t>むぎ歯科</t>
+  </si>
+  <si>
+    <t>2026-09-26</t>
+  </si>
+  <si>
+    <t>はま歯科医院</t>
+  </si>
+  <si>
+    <t>2026-09-11</t>
+  </si>
+  <si>
+    <t>錦糸町矯正歯科クリニック</t>
+  </si>
+  <si>
+    <t>2026-09-07</t>
+  </si>
+  <si>
+    <t>整体処 たくみ堂</t>
+  </si>
+  <si>
+    <t>2026-08-07</t>
+  </si>
+  <si>
+    <t>千歳烏山ケンズ歯科</t>
+  </si>
+  <si>
+    <t>2026-08-03</t>
+  </si>
+  <si>
+    <t>GAJUM photo studio</t>
+  </si>
+  <si>
+    <t>金町駅前ジャスミン歯科</t>
+  </si>
+  <si>
+    <t>ストレッチ&amp;ボディケア m.o.v.e巣鴨店</t>
+  </si>
+  <si>
+    <t>2026-07-30</t>
+  </si>
+  <si>
+    <t>堀田歯科（リンク先変更前）</t>
+  </si>
+  <si>
+    <t>きしかわデンタルオフィス</t>
+  </si>
+  <si>
+    <t>2026-07-27</t>
+  </si>
+  <si>
+    <t>COCORO エステサロン</t>
+  </si>
+  <si>
+    <t>2026-07-21</t>
+  </si>
+  <si>
+    <t>なかはら歯科クリニック</t>
+  </si>
+  <si>
+    <t>住友歯科医院</t>
+  </si>
+  <si>
+    <t>2026-04-02</t>
+  </si>
+  <si>
+    <t>大神宮デンタルクリニック</t>
+  </si>
+  <si>
+    <t>2026-07-16</t>
+  </si>
+  <si>
+    <t>はんだ歯科医院</t>
+  </si>
+  <si>
+    <t>竹内歯科クリニック（審美歯科）</t>
+  </si>
+  <si>
+    <t>2026-07-17</t>
+  </si>
+  <si>
+    <t>銀座トレーニングラボ</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xml:space="preserve">
-  <numFmts count="0"/>
-  <fonts count="2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <fonts count="3" x14ac:knownFonts="1">
     <font>
-      <b val="0"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
     </font>
     <font>
-      <b val="1"/>
-      <i val="0"/>
-      <strike val="0"/>
-      <u val="none"/>
+      <b/>
       <sz val="11"/>
       <color rgb="FF000000"/>
       <name val="Calibri"/>
+    </font>
+    <font>
+      <sz val="6"/>
+      <name val="ＭＳ Ｐゴシック"/>
+      <family val="3"/>
+      <charset val="128"/>
     </font>
   </fonts>
   <fills count="2">
@@ -215,36 +305,36 @@
       <patternFill patternType="none"/>
     </fill>
     <fill>
-      <patternFill patternType="gray125">
-        <fgColor rgb="FFFFFFFF"/>
-        <bgColor rgb="FF000000"/>
-      </patternFill>
+      <patternFill patternType="gray125"/>
     </fill>
   </fills>
   <borders count="1">
-    <border/>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
   <cellXfs count="2">
-    <xf xfId="0" fontId="0" numFmtId="0" fillId="0" borderId="0" applyFont="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
-    <xf xfId="0" fontId="1" numFmtId="0" fillId="0" borderId="0" applyFont="1" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" shrinkToFit="false"/>
-    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="標準" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
-  <tableStyles defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotTableStyle1"/>
+  <tableStyles count="0" defaultTableStyle="TableStyleMedium9"/>
+  <extLst>
+    <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
+      <x14:slicerStyles defaultSlicerStyle="SlicerStyleLight1"/>
+    </ext>
+  </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -533,14 +623,11 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xml:space="preserve">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-  </sheetPr>
-  <dimension ref="A1:Y13"/>
-  <sheetFormatPr defaultRowHeight="14.4" defaultColWidth="20" outlineLevelRow="0" outlineLevelCol="0"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="A1:Y32"/>
+  <sheetFormatPr defaultColWidth="20" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <sheetData>
-    <row r="1" spans="1:25">
+    <row r="1" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -617,7 +704,7 @@
         <v>24</v>
       </c>
     </row>
-    <row r="2" spans="1:25">
+    <row r="2" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A2" t="s">
         <v>25</v>
       </c>
@@ -667,7 +754,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="3" spans="1:25">
+    <row r="3" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A3" t="s">
         <v>25</v>
       </c>
@@ -717,7 +804,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:25">
+    <row r="4" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A4" t="s">
         <v>25</v>
       </c>
@@ -767,7 +854,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="5" spans="1:25">
+    <row r="5" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A5" t="s">
         <v>25</v>
       </c>
@@ -817,7 +904,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="6" spans="1:25">
+    <row r="6" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A6" t="s">
         <v>25</v>
       </c>
@@ -864,34 +951,34 @@
         <v>3164</v>
       </c>
       <c r="P6">
-        <v>1283.817952</v>
+        <v>1283.8179520000001</v>
       </c>
       <c r="Q6">
         <v>78</v>
       </c>
       <c r="S6">
-        <v>52.076923</v>
+        <v>52.076923000000001</v>
       </c>
       <c r="T6">
-        <v>2.465234</v>
+        <v>2.4652340000000001</v>
       </c>
       <c r="U6">
         <v>86</v>
       </c>
       <c r="V6">
-        <v>2.718078</v>
+        <v>2.7180780000000002</v>
       </c>
       <c r="W6">
-        <v>47.232558</v>
+        <v>47.232557999999997</v>
       </c>
       <c r="X6">
         <v>66</v>
       </c>
       <c r="Y6">
-        <v>61.545455</v>
-      </c>
-    </row>
-    <row r="7" spans="1:25">
+        <v>61.545454999999997</v>
+      </c>
+    </row>
+    <row r="7" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A7" t="s">
         <v>25</v>
       </c>
@@ -917,10 +1004,10 @@
         <v>1770</v>
       </c>
       <c r="I7">
-        <v>1.612429</v>
+        <v>1.6124289999999999</v>
       </c>
       <c r="J7">
-        <v>54.98648649</v>
+        <v>54.986486489999997</v>
       </c>
       <c r="K7">
         <v>160</v>
@@ -944,28 +1031,28 @@
         <v>74</v>
       </c>
       <c r="S7">
-        <v>54.986486</v>
+        <v>54.986485999999999</v>
       </c>
       <c r="T7">
-        <v>2.592852</v>
+        <v>2.5928520000000002</v>
       </c>
       <c r="U7">
         <v>79</v>
       </c>
       <c r="V7">
-        <v>2.768045</v>
+        <v>2.7680449999999999</v>
       </c>
       <c r="W7">
-        <v>51.506329</v>
+        <v>51.506329000000001</v>
       </c>
       <c r="X7">
         <v>62</v>
       </c>
       <c r="Y7">
-        <v>65.629032</v>
-      </c>
-    </row>
-    <row r="8" spans="1:25">
+        <v>65.629031999999995</v>
+      </c>
+    </row>
+    <row r="8" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A8" t="s">
         <v>25</v>
       </c>
@@ -994,7 +1081,7 @@
         <v>1.521347</v>
       </c>
       <c r="J8">
-        <v>58.22857143</v>
+        <v>58.228571430000002</v>
       </c>
       <c r="K8">
         <v>160</v>
@@ -1018,7 +1105,7 @@
         <v>70</v>
       </c>
       <c r="S8">
-        <v>58.228571</v>
+        <v>58.228571000000002</v>
       </c>
       <c r="T8">
         <v>2.182725</v>
@@ -1030,16 +1117,16 @@
         <v>2.400998</v>
       </c>
       <c r="W8">
-        <v>52.935065</v>
+        <v>52.935065000000002</v>
       </c>
       <c r="X8">
         <v>58</v>
       </c>
       <c r="Y8">
-        <v>70.275862</v>
-      </c>
-    </row>
-    <row r="9" spans="1:25">
+        <v>70.275862000000004</v>
+      </c>
+    </row>
+    <row r="9" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A9" t="s">
         <v>25</v>
       </c>
@@ -1065,10 +1152,10 @@
         <v>1782</v>
       </c>
       <c r="I9">
-        <v>1.80303</v>
+        <v>1.8030299999999999</v>
       </c>
       <c r="J9">
-        <v>56.33333333</v>
+        <v>56.333333330000002</v>
       </c>
       <c r="K9">
         <v>160</v>
@@ -1092,19 +1179,19 @@
         <v>72</v>
       </c>
       <c r="S9">
-        <v>56.333333</v>
+        <v>56.333333000000003</v>
       </c>
       <c r="T9">
-        <v>2.240896</v>
+        <v>2.2408960000000002</v>
       </c>
       <c r="U9">
         <v>87</v>
       </c>
       <c r="V9">
-        <v>2.70775</v>
+        <v>2.7077499999999999</v>
       </c>
       <c r="W9">
-        <v>46.62069</v>
+        <v>46.620690000000003</v>
       </c>
       <c r="X9">
         <v>64</v>
@@ -1113,7 +1200,7 @@
         <v>63.375</v>
       </c>
     </row>
-    <row r="10" spans="1:25">
+    <row r="10" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A10" t="s">
         <v>25</v>
       </c>
@@ -1142,7 +1229,7 @@
         <v>2.003603</v>
       </c>
       <c r="J10">
-        <v>34.02521008</v>
+        <v>34.025210080000001</v>
       </c>
       <c r="K10">
         <v>160</v>
@@ -1160,16 +1247,16 @@
         <v>3893</v>
       </c>
       <c r="P10">
-        <v>1040.071924</v>
+        <v>1040.0719240000001</v>
       </c>
       <c r="Q10">
         <v>119</v>
       </c>
       <c r="S10">
-        <v>34.02521</v>
+        <v>34.025210000000001</v>
       </c>
       <c r="T10">
-        <v>3.056769</v>
+        <v>3.0567690000000001</v>
       </c>
       <c r="U10">
         <v>142</v>
@@ -1178,16 +1265,16 @@
         <v>3.647573</v>
       </c>
       <c r="W10">
-        <v>28.514085</v>
+        <v>28.514085000000001</v>
       </c>
       <c r="X10">
         <v>103</v>
       </c>
       <c r="Y10">
-        <v>39.31068</v>
-      </c>
-    </row>
-    <row r="11" spans="1:25">
+        <v>39.310679999999998</v>
+      </c>
+    </row>
+    <row r="11" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A11" t="s">
         <v>25</v>
       </c>
@@ -1216,7 +1303,7 @@
         <v>1.447484</v>
       </c>
       <c r="J11">
-        <v>56.54166667</v>
+        <v>56.541666669999998</v>
       </c>
       <c r="K11">
         <v>160</v>
@@ -1240,7 +1327,7 @@
         <v>72</v>
       </c>
       <c r="S11">
-        <v>56.541667</v>
+        <v>56.541666999999997</v>
       </c>
       <c r="T11">
         <v>2.721088</v>
@@ -1252,16 +1339,16 @@
         <v>3.287982</v>
       </c>
       <c r="W11">
-        <v>46.793103</v>
+        <v>46.793103000000002</v>
       </c>
       <c r="X11">
         <v>62</v>
       </c>
       <c r="Y11">
-        <v>65.66129</v>
-      </c>
-    </row>
-    <row r="12" spans="1:25">
+        <v>65.661289999999994</v>
+      </c>
+    </row>
+    <row r="12" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A12" t="s">
         <v>25</v>
       </c>
@@ -1287,7 +1374,7 @@
         <v>2248</v>
       </c>
       <c r="I12">
-        <v>1.476868</v>
+        <v>1.4768680000000001</v>
       </c>
       <c r="J12">
         <v>23.125</v>
@@ -1308,7 +1395,7 @@
         <v>3320</v>
       </c>
       <c r="P12">
-        <v>835.843373</v>
+        <v>835.84337300000004</v>
       </c>
       <c r="Q12">
         <v>120</v>
@@ -1317,25 +1404,25 @@
         <v>23.125</v>
       </c>
       <c r="T12">
-        <v>3.614458</v>
+        <v>3.6144579999999999</v>
       </c>
       <c r="U12">
         <v>136</v>
       </c>
       <c r="V12">
-        <v>4.096386</v>
+        <v>4.0963859999999999</v>
       </c>
       <c r="W12">
-        <v>20.404412</v>
+        <v>20.404412000000001</v>
       </c>
       <c r="X12">
         <v>112</v>
       </c>
       <c r="Y12">
-        <v>24.776786</v>
-      </c>
-    </row>
-    <row r="13" spans="1:25">
+        <v>24.776786000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:25" x14ac:dyDescent="0.3">
       <c r="A13" t="s">
         <v>25</v>
       </c>
@@ -1364,7 +1451,7 @@
         <v>1.0125</v>
       </c>
       <c r="J13">
-        <v>26.33333333</v>
+        <v>26.333333329999999</v>
       </c>
       <c r="K13" t="s">
         <v>34</v>
@@ -1382,7 +1469,7 @@
         <v>81</v>
       </c>
       <c r="P13">
-        <v>975.308642</v>
+        <v>975.30864199999996</v>
       </c>
       <c r="Q13">
         <v>4</v>
@@ -1391,13 +1478,13 @@
         <v>19.75</v>
       </c>
       <c r="T13">
-        <v>4.938272</v>
+        <v>4.9382720000000004</v>
       </c>
       <c r="U13">
         <v>4</v>
       </c>
       <c r="V13">
-        <v>4.938272</v>
+        <v>4.9382720000000004</v>
       </c>
       <c r="W13">
         <v>19.75</v>
@@ -1409,18 +1496,1368 @@
         <v>26.333333</v>
       </c>
     </row>
+    <row r="14" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A14" t="s">
+        <v>25</v>
+      </c>
+      <c r="B14" t="s">
+        <v>26</v>
+      </c>
+      <c r="C14" t="s">
+        <v>84</v>
+      </c>
+      <c r="D14" t="s">
+        <v>38</v>
+      </c>
+      <c r="E14" t="s">
+        <v>29</v>
+      </c>
+      <c r="F14">
+        <v>59</v>
+      </c>
+      <c r="G14" t="s">
+        <v>42</v>
+      </c>
+      <c r="H14">
+        <v>1870</v>
+      </c>
+      <c r="I14">
+        <v>3.5294120000000002</v>
+      </c>
+      <c r="J14">
+        <v>96.542372880000002</v>
+      </c>
+      <c r="K14" t="s">
+        <v>34</v>
+      </c>
+      <c r="L14">
+        <v>0</v>
+      </c>
+      <c r="M14">
+        <v>5696</v>
+      </c>
+      <c r="N14" t="s">
+        <v>35</v>
+      </c>
+      <c r="O14">
+        <v>6600</v>
+      </c>
+      <c r="P14">
+        <v>863.030303</v>
+      </c>
+      <c r="Q14">
+        <v>59</v>
+      </c>
+      <c r="S14">
+        <v>96.542372999999998</v>
+      </c>
+      <c r="T14">
+        <v>0.89393900000000004</v>
+      </c>
+      <c r="U14">
+        <v>63</v>
+      </c>
+      <c r="V14">
+        <v>0.95454499999999998</v>
+      </c>
+      <c r="W14">
+        <v>90.412698000000006</v>
+      </c>
+    </row>
+    <row r="15" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A15" t="s">
+        <v>25</v>
+      </c>
+      <c r="B15" t="s">
+        <v>26</v>
+      </c>
+      <c r="C15" t="s">
+        <v>32</v>
+      </c>
+      <c r="D15" t="s">
+        <v>38</v>
+      </c>
+      <c r="E15" t="s">
+        <v>29</v>
+      </c>
+      <c r="F15">
+        <v>76</v>
+      </c>
+      <c r="G15" t="s">
+        <v>42</v>
+      </c>
+      <c r="H15">
+        <v>4541</v>
+      </c>
+      <c r="I15">
+        <v>1.30566</v>
+      </c>
+      <c r="J15">
+        <v>80.53947368</v>
+      </c>
+      <c r="K15" t="s">
+        <v>34</v>
+      </c>
+      <c r="L15">
+        <v>0</v>
+      </c>
+      <c r="M15">
+        <v>6121</v>
+      </c>
+      <c r="N15" t="s">
+        <v>83</v>
+      </c>
+      <c r="O15">
+        <v>5929</v>
+      </c>
+      <c r="P15">
+        <v>1032.3832010000001</v>
+      </c>
+      <c r="Q15">
+        <v>76</v>
+      </c>
+      <c r="S15">
+        <v>80.539473999999998</v>
+      </c>
+      <c r="T15">
+        <v>1.2818350000000001</v>
+      </c>
+      <c r="U15">
+        <v>80</v>
+      </c>
+      <c r="V15">
+        <v>1.3492999999999999</v>
+      </c>
+      <c r="W15">
+        <v>76.512500000000003</v>
+      </c>
+    </row>
+    <row r="16" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A16" t="s">
+        <v>25</v>
+      </c>
+      <c r="B16" t="s">
+        <v>26</v>
+      </c>
+      <c r="C16" t="s">
+        <v>82</v>
+      </c>
+      <c r="D16" t="s">
+        <v>38</v>
+      </c>
+      <c r="E16" t="s">
+        <v>29</v>
+      </c>
+      <c r="F16">
+        <v>90</v>
+      </c>
+      <c r="G16" t="s">
+        <v>42</v>
+      </c>
+      <c r="H16">
+        <v>4227</v>
+      </c>
+      <c r="I16">
+        <v>1.2893300000000001</v>
+      </c>
+      <c r="J16">
+        <v>69.844444440000004</v>
+      </c>
+      <c r="K16" t="s">
+        <v>34</v>
+      </c>
+      <c r="L16">
+        <v>0</v>
+      </c>
+      <c r="M16">
+        <v>6286</v>
+      </c>
+      <c r="N16" t="s">
+        <v>80</v>
+      </c>
+      <c r="O16">
+        <v>5450</v>
+      </c>
+      <c r="P16">
+        <v>1153.394495</v>
+      </c>
+      <c r="Q16">
+        <v>90</v>
+      </c>
+      <c r="S16">
+        <v>69.844443999999996</v>
+      </c>
+      <c r="T16">
+        <v>1.651376</v>
+      </c>
+      <c r="U16">
+        <v>101</v>
+      </c>
+      <c r="V16">
+        <v>1.8532109999999999</v>
+      </c>
+      <c r="W16">
+        <v>62.237623999999997</v>
+      </c>
+    </row>
+    <row r="17" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A17" t="s">
+        <v>25</v>
+      </c>
+      <c r="B17" t="s">
+        <v>26</v>
+      </c>
+      <c r="C17" t="s">
+        <v>81</v>
+      </c>
+      <c r="D17" t="s">
+        <v>38</v>
+      </c>
+      <c r="E17" t="s">
+        <v>29</v>
+      </c>
+      <c r="F17">
+        <v>341</v>
+      </c>
+      <c r="G17" t="s">
+        <v>42</v>
+      </c>
+      <c r="H17">
+        <v>4068</v>
+      </c>
+      <c r="I17">
+        <v>1.308997</v>
+      </c>
+      <c r="J17">
+        <v>17.630498530000001</v>
+      </c>
+      <c r="K17" t="s">
+        <v>34</v>
+      </c>
+      <c r="L17">
+        <v>0</v>
+      </c>
+      <c r="M17">
+        <v>6012</v>
+      </c>
+      <c r="N17" t="s">
+        <v>80</v>
+      </c>
+      <c r="O17">
+        <v>5325</v>
+      </c>
+      <c r="P17">
+        <v>1129.014085</v>
+      </c>
+      <c r="Q17">
+        <v>341</v>
+      </c>
+      <c r="S17">
+        <v>17.630499</v>
+      </c>
+      <c r="T17">
+        <v>6.4037559999999996</v>
+      </c>
+      <c r="U17">
+        <v>354</v>
+      </c>
+      <c r="V17">
+        <v>6.6478869999999999</v>
+      </c>
+      <c r="W17">
+        <v>16.983051</v>
+      </c>
+    </row>
+    <row r="18" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A18" t="s">
+        <v>25</v>
+      </c>
+      <c r="B18" t="s">
+        <v>26</v>
+      </c>
+      <c r="C18" t="s">
+        <v>79</v>
+      </c>
+      <c r="D18" t="s">
+        <v>28</v>
+      </c>
+      <c r="E18" t="s">
+        <v>29</v>
+      </c>
+      <c r="F18">
+        <v>131</v>
+      </c>
+      <c r="G18" t="s">
+        <v>42</v>
+      </c>
+      <c r="H18">
+        <v>3654</v>
+      </c>
+      <c r="I18">
+        <v>1.4731799999999999</v>
+      </c>
+      <c r="J18">
+        <v>48.671755730000001</v>
+      </c>
+      <c r="K18" t="s">
+        <v>34</v>
+      </c>
+      <c r="L18">
+        <v>0</v>
+      </c>
+      <c r="M18">
+        <v>6376</v>
+      </c>
+      <c r="N18" t="s">
+        <v>78</v>
+      </c>
+      <c r="O18">
+        <v>5383</v>
+      </c>
+      <c r="P18">
+        <v>1184.4696269999999</v>
+      </c>
+      <c r="Q18">
+        <v>131</v>
+      </c>
+      <c r="S18">
+        <v>48.671756000000002</v>
+      </c>
+      <c r="T18">
+        <v>2.4335870000000002</v>
+      </c>
+      <c r="U18">
+        <v>134</v>
+      </c>
+      <c r="V18">
+        <v>2.4893179999999999</v>
+      </c>
+      <c r="W18">
+        <v>47.582090000000001</v>
+      </c>
+    </row>
+    <row r="19" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A19" t="s">
+        <v>25</v>
+      </c>
+      <c r="B19" t="s">
+        <v>26</v>
+      </c>
+      <c r="C19" t="s">
+        <v>77</v>
+      </c>
+      <c r="D19" t="s">
+        <v>38</v>
+      </c>
+      <c r="E19" t="s">
+        <v>29</v>
+      </c>
+      <c r="F19">
+        <v>139</v>
+      </c>
+      <c r="G19" t="s">
+        <v>42</v>
+      </c>
+      <c r="H19">
+        <v>3867</v>
+      </c>
+      <c r="I19">
+        <v>1.566589</v>
+      </c>
+      <c r="J19">
+        <v>44.64028777</v>
+      </c>
+      <c r="K19" t="s">
+        <v>34</v>
+      </c>
+      <c r="L19">
+        <v>0</v>
+      </c>
+      <c r="M19">
+        <v>6205</v>
+      </c>
+      <c r="N19" t="s">
+        <v>75</v>
+      </c>
+      <c r="O19">
+        <v>6058</v>
+      </c>
+      <c r="P19">
+        <v>1024.2654339999999</v>
+      </c>
+      <c r="Q19">
+        <v>139</v>
+      </c>
+      <c r="S19">
+        <v>44.640287999999998</v>
+      </c>
+      <c r="T19">
+        <v>2.2944870000000002</v>
+      </c>
+      <c r="U19">
+        <v>153</v>
+      </c>
+      <c r="V19">
+        <v>2.5255860000000001</v>
+      </c>
+      <c r="W19">
+        <v>40.555556000000003</v>
+      </c>
+    </row>
+    <row r="20" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A20" t="s">
+        <v>25</v>
+      </c>
+      <c r="B20" t="s">
+        <v>26</v>
+      </c>
+      <c r="C20" t="s">
+        <v>76</v>
+      </c>
+      <c r="D20" t="s">
+        <v>38</v>
+      </c>
+      <c r="E20" t="s">
+        <v>29</v>
+      </c>
+      <c r="F20">
+        <v>191</v>
+      </c>
+      <c r="G20" t="s">
+        <v>42</v>
+      </c>
+      <c r="H20">
+        <v>3867</v>
+      </c>
+      <c r="I20">
+        <v>1.3935869999999999</v>
+      </c>
+      <c r="J20">
+        <v>31.570680629999998</v>
+      </c>
+      <c r="K20" t="s">
+        <v>34</v>
+      </c>
+      <c r="L20">
+        <v>0</v>
+      </c>
+      <c r="M20">
+        <v>6030</v>
+      </c>
+      <c r="N20" t="s">
+        <v>75</v>
+      </c>
+      <c r="O20">
+        <v>5389</v>
+      </c>
+      <c r="P20">
+        <v>1118.946001</v>
+      </c>
+      <c r="Q20">
+        <v>191</v>
+      </c>
+      <c r="S20">
+        <v>31.570681</v>
+      </c>
+      <c r="T20">
+        <v>3.544257</v>
+      </c>
+      <c r="U20">
+        <v>196</v>
+      </c>
+      <c r="V20">
+        <v>3.637038</v>
+      </c>
+      <c r="W20">
+        <v>30.765305999999999</v>
+      </c>
+    </row>
+    <row r="21" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A21" t="s">
+        <v>25</v>
+      </c>
+      <c r="B21" t="s">
+        <v>26</v>
+      </c>
+      <c r="C21" t="s">
+        <v>74</v>
+      </c>
+      <c r="D21" t="s">
+        <v>38</v>
+      </c>
+      <c r="E21" t="s">
+        <v>29</v>
+      </c>
+      <c r="F21">
+        <v>158</v>
+      </c>
+      <c r="G21" t="s">
+        <v>42</v>
+      </c>
+      <c r="H21">
+        <v>2772</v>
+      </c>
+      <c r="I21">
+        <v>1.425325</v>
+      </c>
+      <c r="J21">
+        <v>42.575949369999996</v>
+      </c>
+      <c r="K21" t="s">
+        <v>34</v>
+      </c>
+      <c r="L21">
+        <v>0</v>
+      </c>
+      <c r="M21">
+        <v>6727</v>
+      </c>
+      <c r="N21" t="s">
+        <v>73</v>
+      </c>
+      <c r="O21">
+        <v>3951</v>
+      </c>
+      <c r="P21">
+        <v>1702.606935</v>
+      </c>
+      <c r="Q21">
+        <v>158</v>
+      </c>
+      <c r="S21">
+        <v>42.575949000000001</v>
+      </c>
+      <c r="T21">
+        <v>3.9989880000000002</v>
+      </c>
+      <c r="U21">
+        <v>172</v>
+      </c>
+      <c r="V21">
+        <v>4.3533280000000003</v>
+      </c>
+      <c r="W21">
+        <v>39.110464999999998</v>
+      </c>
+    </row>
+    <row r="22" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A22" t="s">
+        <v>25</v>
+      </c>
+      <c r="B22" t="s">
+        <v>26</v>
+      </c>
+      <c r="C22" t="s">
+        <v>72</v>
+      </c>
+      <c r="D22" t="s">
+        <v>28</v>
+      </c>
+      <c r="E22" t="s">
+        <v>29</v>
+      </c>
+      <c r="F22">
+        <v>130</v>
+      </c>
+      <c r="G22" t="s">
+        <v>42</v>
+      </c>
+      <c r="H22">
+        <v>3345</v>
+      </c>
+      <c r="I22">
+        <v>1.252616</v>
+      </c>
+      <c r="J22">
+        <v>51.984615380000001</v>
+      </c>
+      <c r="K22" t="s">
+        <v>34</v>
+      </c>
+      <c r="L22">
+        <v>0</v>
+      </c>
+      <c r="M22">
+        <v>6758</v>
+      </c>
+      <c r="N22" t="s">
+        <v>70</v>
+      </c>
+      <c r="O22">
+        <v>4190</v>
+      </c>
+      <c r="P22">
+        <v>1612.8878279999999</v>
+      </c>
+      <c r="Q22">
+        <v>130</v>
+      </c>
+      <c r="S22">
+        <v>51.984614999999998</v>
+      </c>
+      <c r="T22">
+        <v>3.1026250000000002</v>
+      </c>
+      <c r="U22">
+        <v>139</v>
+      </c>
+      <c r="V22">
+        <v>3.3174220000000001</v>
+      </c>
+      <c r="W22">
+        <v>48.618704999999999</v>
+      </c>
+      <c r="X22">
+        <v>61</v>
+      </c>
+      <c r="Y22">
+        <v>110.786885</v>
+      </c>
+    </row>
+    <row r="23" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A23" t="s">
+        <v>25</v>
+      </c>
+      <c r="B23" t="s">
+        <v>26</v>
+      </c>
+      <c r="C23" t="s">
+        <v>71</v>
+      </c>
+      <c r="D23" t="s">
+        <v>28</v>
+      </c>
+      <c r="E23" t="s">
+        <v>29</v>
+      </c>
+      <c r="F23">
+        <v>164</v>
+      </c>
+      <c r="G23" t="s">
+        <v>42</v>
+      </c>
+      <c r="H23">
+        <v>3996</v>
+      </c>
+      <c r="I23">
+        <v>1.2777780000000001</v>
+      </c>
+      <c r="J23">
+        <v>40.237804879999999</v>
+      </c>
+      <c r="K23" t="s">
+        <v>34</v>
+      </c>
+      <c r="L23">
+        <v>0</v>
+      </c>
+      <c r="M23">
+        <v>6599</v>
+      </c>
+      <c r="N23" t="s">
+        <v>70</v>
+      </c>
+      <c r="O23">
+        <v>5106</v>
+      </c>
+      <c r="P23">
+        <v>1292.4010969999999</v>
+      </c>
+      <c r="Q23">
+        <v>164</v>
+      </c>
+      <c r="S23">
+        <v>40.237805000000002</v>
+      </c>
+      <c r="T23">
+        <v>3.2119080000000002</v>
+      </c>
+      <c r="U23">
+        <v>168</v>
+      </c>
+      <c r="V23">
+        <v>3.2902469999999999</v>
+      </c>
+      <c r="W23">
+        <v>39.279761999999998</v>
+      </c>
+      <c r="X23">
+        <v>138</v>
+      </c>
+      <c r="Y23">
+        <v>47.818840999999999</v>
+      </c>
+    </row>
+    <row r="24" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A24" t="s">
+        <v>25</v>
+      </c>
+      <c r="B24" t="s">
+        <v>26</v>
+      </c>
+      <c r="C24" t="s">
+        <v>69</v>
+      </c>
+      <c r="D24" t="s">
+        <v>38</v>
+      </c>
+      <c r="E24" t="s">
+        <v>29</v>
+      </c>
+      <c r="F24">
+        <v>156</v>
+      </c>
+      <c r="G24" t="s">
+        <v>42</v>
+      </c>
+      <c r="H24">
+        <v>3821</v>
+      </c>
+      <c r="I24">
+        <v>1.432348</v>
+      </c>
+      <c r="J24">
+        <v>40.493589739999997</v>
+      </c>
+      <c r="K24" t="s">
+        <v>34</v>
+      </c>
+      <c r="L24">
+        <v>0</v>
+      </c>
+      <c r="M24">
+        <v>6317</v>
+      </c>
+      <c r="N24" t="s">
+        <v>66</v>
+      </c>
+      <c r="O24">
+        <v>5473</v>
+      </c>
+      <c r="P24">
+        <v>1154.2115839999999</v>
+      </c>
+      <c r="Q24">
+        <v>156</v>
+      </c>
+      <c r="S24">
+        <v>40.493589999999998</v>
+      </c>
+      <c r="T24">
+        <v>2.8503560000000001</v>
+      </c>
+      <c r="U24">
+        <v>180</v>
+      </c>
+      <c r="V24">
+        <v>3.2888730000000002</v>
+      </c>
+      <c r="W24">
+        <v>35.094444000000003</v>
+      </c>
+      <c r="X24">
+        <v>127</v>
+      </c>
+      <c r="Y24">
+        <v>49.740157000000004</v>
+      </c>
+    </row>
+    <row r="25" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A25" t="s">
+        <v>25</v>
+      </c>
+      <c r="B25" t="s">
+        <v>26</v>
+      </c>
+      <c r="C25" t="s">
+        <v>68</v>
+      </c>
+      <c r="D25" t="s">
+        <v>28</v>
+      </c>
+      <c r="E25" t="s">
+        <v>29</v>
+      </c>
+      <c r="F25">
+        <v>104</v>
+      </c>
+      <c r="G25" t="s">
+        <v>42</v>
+      </c>
+      <c r="H25">
+        <v>3131</v>
+      </c>
+      <c r="I25">
+        <v>1.4484189999999999</v>
+      </c>
+      <c r="J25">
+        <v>38.75</v>
+      </c>
+      <c r="K25" t="s">
+        <v>34</v>
+      </c>
+      <c r="L25">
+        <v>0</v>
+      </c>
+      <c r="M25">
+        <v>4030</v>
+      </c>
+      <c r="N25" t="s">
+        <v>26</v>
+      </c>
+      <c r="O25">
+        <v>4535</v>
+      </c>
+      <c r="P25">
+        <v>888.64388099999996</v>
+      </c>
+      <c r="Q25">
+        <v>104</v>
+      </c>
+      <c r="S25">
+        <v>38.75</v>
+      </c>
+      <c r="T25">
+        <v>2.293275</v>
+      </c>
+      <c r="U25">
+        <v>125</v>
+      </c>
+      <c r="V25">
+        <v>2.7563399999999998</v>
+      </c>
+      <c r="W25">
+        <v>32.24</v>
+      </c>
+      <c r="X25">
+        <v>91</v>
+      </c>
+      <c r="Y25">
+        <v>44.285713999999999</v>
+      </c>
+    </row>
+    <row r="26" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A26" t="s">
+        <v>25</v>
+      </c>
+      <c r="B26" t="s">
+        <v>26</v>
+      </c>
+      <c r="C26" t="s">
+        <v>67</v>
+      </c>
+      <c r="D26" t="s">
+        <v>38</v>
+      </c>
+      <c r="E26" t="s">
+        <v>29</v>
+      </c>
+      <c r="F26">
+        <v>97</v>
+      </c>
+      <c r="G26" t="s">
+        <v>42</v>
+      </c>
+      <c r="H26">
+        <v>6350</v>
+      </c>
+      <c r="I26">
+        <v>1.571496</v>
+      </c>
+      <c r="J26">
+        <v>64.288659789999997</v>
+      </c>
+      <c r="K26" t="s">
+        <v>34</v>
+      </c>
+      <c r="L26">
+        <v>0</v>
+      </c>
+      <c r="M26">
+        <v>6236</v>
+      </c>
+      <c r="N26" t="s">
+        <v>66</v>
+      </c>
+      <c r="O26">
+        <v>9979</v>
+      </c>
+      <c r="P26">
+        <v>624.91231600000003</v>
+      </c>
+      <c r="Q26">
+        <v>97</v>
+      </c>
+      <c r="S26">
+        <v>64.288659999999993</v>
+      </c>
+      <c r="T26">
+        <v>0.97204100000000004</v>
+      </c>
+      <c r="U26">
+        <v>106</v>
+      </c>
+      <c r="V26">
+        <v>1.0622309999999999</v>
+      </c>
+      <c r="W26">
+        <v>58.830188999999997</v>
+      </c>
+      <c r="X26">
+        <v>69</v>
+      </c>
+      <c r="Y26">
+        <v>90.376812000000001</v>
+      </c>
+    </row>
+    <row r="27" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A27" t="s">
+        <v>25</v>
+      </c>
+      <c r="B27" t="s">
+        <v>26</v>
+      </c>
+      <c r="C27" t="s">
+        <v>65</v>
+      </c>
+      <c r="D27" t="s">
+        <v>38</v>
+      </c>
+      <c r="E27" t="s">
+        <v>29</v>
+      </c>
+      <c r="F27">
+        <v>133</v>
+      </c>
+      <c r="G27" t="s">
+        <v>42</v>
+      </c>
+      <c r="H27">
+        <v>5249</v>
+      </c>
+      <c r="I27">
+        <v>1.5223850000000001</v>
+      </c>
+      <c r="J27">
+        <v>47.127819549999998</v>
+      </c>
+      <c r="K27" t="s">
+        <v>34</v>
+      </c>
+      <c r="L27">
+        <v>0</v>
+      </c>
+      <c r="M27">
+        <v>6268</v>
+      </c>
+      <c r="N27" t="s">
+        <v>64</v>
+      </c>
+      <c r="O27">
+        <v>7991</v>
+      </c>
+      <c r="P27">
+        <v>784.38243</v>
+      </c>
+      <c r="Q27">
+        <v>133</v>
+      </c>
+      <c r="S27">
+        <v>47.12782</v>
+      </c>
+      <c r="T27">
+        <v>1.664372</v>
+      </c>
+      <c r="U27">
+        <v>141</v>
+      </c>
+      <c r="V27">
+        <v>1.7644850000000001</v>
+      </c>
+      <c r="W27">
+        <v>44.453901000000002</v>
+      </c>
+      <c r="X27">
+        <v>90</v>
+      </c>
+      <c r="Y27">
+        <v>69.644443999999993</v>
+      </c>
+    </row>
+    <row r="28" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A28" t="s">
+        <v>25</v>
+      </c>
+      <c r="B28" t="s">
+        <v>26</v>
+      </c>
+      <c r="C28" t="s">
+        <v>63</v>
+      </c>
+      <c r="D28" t="s">
+        <v>41</v>
+      </c>
+      <c r="E28" t="s">
+        <v>29</v>
+      </c>
+      <c r="F28">
+        <v>133</v>
+      </c>
+      <c r="G28" t="s">
+        <v>42</v>
+      </c>
+      <c r="H28">
+        <v>2723</v>
+      </c>
+      <c r="I28">
+        <v>1.345575</v>
+      </c>
+      <c r="J28">
+        <v>50.751879700000003</v>
+      </c>
+      <c r="K28" t="s">
+        <v>34</v>
+      </c>
+      <c r="L28">
+        <v>0</v>
+      </c>
+      <c r="M28">
+        <v>6750</v>
+      </c>
+      <c r="N28" t="s">
+        <v>62</v>
+      </c>
+      <c r="O28">
+        <v>3664</v>
+      </c>
+      <c r="P28">
+        <v>1842.248908</v>
+      </c>
+      <c r="Q28">
+        <v>133</v>
+      </c>
+      <c r="S28">
+        <v>50.75188</v>
+      </c>
+      <c r="T28">
+        <v>3.6299130000000002</v>
+      </c>
+      <c r="U28">
+        <v>153</v>
+      </c>
+      <c r="V28">
+        <v>4.175764</v>
+      </c>
+      <c r="W28">
+        <v>44.117646999999998</v>
+      </c>
+      <c r="X28">
+        <v>5</v>
+      </c>
+      <c r="Y28">
+        <v>1350</v>
+      </c>
+    </row>
+    <row r="29" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A29" t="s">
+        <v>25</v>
+      </c>
+      <c r="B29" t="s">
+        <v>26</v>
+      </c>
+      <c r="C29" t="s">
+        <v>61</v>
+      </c>
+      <c r="D29" t="s">
+        <v>28</v>
+      </c>
+      <c r="E29" t="s">
+        <v>29</v>
+      </c>
+      <c r="F29">
+        <v>393</v>
+      </c>
+      <c r="G29" t="s">
+        <v>42</v>
+      </c>
+      <c r="H29">
+        <v>4674</v>
+      </c>
+      <c r="I29">
+        <v>1.629867</v>
+      </c>
+      <c r="J29">
+        <v>14.704834610000001</v>
+      </c>
+      <c r="K29" t="s">
+        <v>34</v>
+      </c>
+      <c r="L29">
+        <v>0</v>
+      </c>
+      <c r="M29">
+        <v>5779</v>
+      </c>
+      <c r="N29" t="s">
+        <v>60</v>
+      </c>
+      <c r="O29">
+        <v>7618</v>
+      </c>
+      <c r="P29">
+        <v>758.59805700000004</v>
+      </c>
+      <c r="Q29">
+        <v>393</v>
+      </c>
+      <c r="S29">
+        <v>14.704834999999999</v>
+      </c>
+      <c r="T29">
+        <v>5.1588339999999997</v>
+      </c>
+      <c r="U29">
+        <v>473</v>
+      </c>
+      <c r="V29">
+        <v>6.2089790000000002</v>
+      </c>
+      <c r="W29">
+        <v>12.217758999999999</v>
+      </c>
+      <c r="X29">
+        <v>328</v>
+      </c>
+      <c r="Y29">
+        <v>17.618901999999999</v>
+      </c>
+    </row>
+    <row r="30" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A30" t="s">
+        <v>25</v>
+      </c>
+      <c r="B30" t="s">
+        <v>26</v>
+      </c>
+      <c r="C30" t="s">
+        <v>59</v>
+      </c>
+      <c r="D30" t="s">
+        <v>41</v>
+      </c>
+      <c r="E30" t="s">
+        <v>29</v>
+      </c>
+      <c r="F30">
+        <v>112</v>
+      </c>
+      <c r="G30" t="s">
+        <v>42</v>
+      </c>
+      <c r="H30">
+        <v>5372</v>
+      </c>
+      <c r="I30">
+        <v>1.556962</v>
+      </c>
+      <c r="J30">
+        <v>57.982142860000003</v>
+      </c>
+      <c r="K30" t="s">
+        <v>34</v>
+      </c>
+      <c r="L30">
+        <v>0</v>
+      </c>
+      <c r="M30">
+        <v>6494</v>
+      </c>
+      <c r="N30" t="s">
+        <v>58</v>
+      </c>
+      <c r="O30">
+        <v>8364</v>
+      </c>
+      <c r="P30">
+        <v>776.42276400000003</v>
+      </c>
+      <c r="Q30">
+        <v>112</v>
+      </c>
+      <c r="S30">
+        <v>57.982143000000001</v>
+      </c>
+      <c r="T30">
+        <v>1.339072</v>
+      </c>
+      <c r="U30">
+        <v>115</v>
+      </c>
+      <c r="V30">
+        <v>1.3749400000000001</v>
+      </c>
+      <c r="W30">
+        <v>56.469565000000003</v>
+      </c>
+      <c r="X30">
+        <v>62</v>
+      </c>
+      <c r="Y30">
+        <v>104.741935</v>
+      </c>
+    </row>
+    <row r="31" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A31" t="s">
+        <v>25</v>
+      </c>
+      <c r="B31" t="s">
+        <v>26</v>
+      </c>
+      <c r="C31" t="s">
+        <v>57</v>
+      </c>
+      <c r="D31" t="s">
+        <v>41</v>
+      </c>
+      <c r="E31" t="s">
+        <v>29</v>
+      </c>
+      <c r="F31">
+        <v>201</v>
+      </c>
+      <c r="G31" t="s">
+        <v>42</v>
+      </c>
+      <c r="H31">
+        <v>3770</v>
+      </c>
+      <c r="I31">
+        <v>1.6358090000000001</v>
+      </c>
+      <c r="J31">
+        <v>30.592039799999998</v>
+      </c>
+      <c r="K31" t="s">
+        <v>34</v>
+      </c>
+      <c r="L31">
+        <v>0</v>
+      </c>
+      <c r="M31">
+        <v>6149</v>
+      </c>
+      <c r="N31" t="s">
+        <v>56</v>
+      </c>
+      <c r="O31">
+        <v>6167</v>
+      </c>
+      <c r="P31">
+        <v>997.08123899999998</v>
+      </c>
+      <c r="Q31">
+        <v>201</v>
+      </c>
+      <c r="S31">
+        <v>30.592040000000001</v>
+      </c>
+      <c r="T31">
+        <v>3.2592829999999999</v>
+      </c>
+      <c r="U31">
+        <v>221</v>
+      </c>
+      <c r="V31">
+        <v>3.5835900000000001</v>
+      </c>
+      <c r="W31">
+        <v>27.823529000000001</v>
+      </c>
+      <c r="X31">
+        <v>179</v>
+      </c>
+      <c r="Y31">
+        <v>34.351954999999997</v>
+      </c>
+    </row>
+    <row r="32" spans="1:25" x14ac:dyDescent="0.3">
+      <c r="A32" t="s">
+        <v>25</v>
+      </c>
+      <c r="B32" t="s">
+        <v>26</v>
+      </c>
+      <c r="C32" t="s">
+        <v>55</v>
+      </c>
+      <c r="D32" t="s">
+        <v>41</v>
+      </c>
+      <c r="E32" t="s">
+        <v>29</v>
+      </c>
+      <c r="F32">
+        <v>154</v>
+      </c>
+      <c r="G32" t="s">
+        <v>42</v>
+      </c>
+      <c r="H32">
+        <v>4251</v>
+      </c>
+      <c r="I32">
+        <v>1.7565280000000001</v>
+      </c>
+      <c r="J32">
+        <v>35.954545449999998</v>
+      </c>
+      <c r="K32" t="s">
+        <v>34</v>
+      </c>
+      <c r="L32">
+        <v>0</v>
+      </c>
+      <c r="M32">
+        <v>5537</v>
+      </c>
+      <c r="N32" t="s">
+        <v>54</v>
+      </c>
+      <c r="O32">
+        <v>7467</v>
+      </c>
+      <c r="P32">
+        <v>741.52939600000002</v>
+      </c>
+      <c r="Q32">
+        <v>154</v>
+      </c>
+      <c r="S32">
+        <v>35.954545000000003</v>
+      </c>
+      <c r="T32">
+        <v>2.062408</v>
+      </c>
+      <c r="U32">
+        <v>206</v>
+      </c>
+      <c r="V32">
+        <v>2.7588050000000002</v>
+      </c>
+      <c r="W32">
+        <v>26.878640999999998</v>
+      </c>
+      <c r="X32">
+        <v>131</v>
+      </c>
+      <c r="Y32">
+        <v>42.267175999999999</v>
+      </c>
+    </row>
   </sheetData>
-  <sheetProtection sheet="false" objects="false" scenarios="false" formatCells="false" formatColumns="false" formatRows="false" insertColumns="false" insertRows="false" insertHyperlinks="false" deleteColumns="false" deleteRows="false" selectLockedCells="false" sort="false" autoFilter="false" pivotTables="false" selectUnlockedCells="false"/>
-  <printOptions gridLines="false" gridLinesSet="true"/>
+  <sheetProtection formatCells="0" formatColumns="0" formatRows="0" insertColumns="0" insertRows="0" insertHyperlinks="0" deleteColumns="0" deleteRows="0" sort="0" autoFilter="0" pivotTables="0"/>
+  <phoneticPr fontId="2"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <pageSetup paperSize="1" orientation="default" scale="100" fitToHeight="1" fitToWidth="1"/>
-  <headerFooter differentOddEven="false" differentFirst="false" scaleWithDoc="true" alignWithMargins="true">
-    <oddHeader/>
-    <oddFooter/>
-    <evenHeader/>
-    <evenFooter/>
-    <firstHeader/>
-    <firstFooter/>
-  </headerFooter>
+  <pageSetup orientation="portrait" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>